<commit_message>
fix: pipeline working and accurecy of ocr
</commit_message>
<xml_diff>
--- a/export_results/evaluation_report.xlsx
+++ b/export_results/evaluation_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,16 +438,64 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8.35</v>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="C3" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6.52</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="C4" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6.15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="n">
-        <v>0</v>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>21.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>